<commit_message>
Began work on textures and normals Signed-off-by: Student Harvey Smith (TL_KCOMP_B_Y3) <t00264389@mymtu.ie>
</commit_message>
<xml_diff>
--- a/Computer Graphics/Computer Graphics - Harvey Smith.xlsx
+++ b/Computer Graphics/Computer Graphics - Harvey Smith.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\StudentHarveySmith(T\Desktop\Comp\Computer Graphics\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\StudentHarveySmith(T\Desktop\CG\Computer Graphics\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="16" documentId="8_{C4E8EF18-1AEB-4960-A7F5-7E91770FD457}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3F8A0CF7-DFEE-48D1-849B-4B623247243B}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC83CC33-9A3F-4416-A3F4-B0CB175B516E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{DD62BD67-B11E-4023-A63C-9D57BBE8FCA5}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="10">
   <si>
     <t>X</t>
   </si>
@@ -60,6 +60,15 @@
   </si>
   <si>
     <t>Back Face</t>
+  </si>
+  <si>
+    <t>RAW</t>
+  </si>
+  <si>
+    <t>PX</t>
+  </si>
+  <si>
+    <t>PY</t>
   </si>
 </sst>
 </file>
@@ -491,6 +500,50 @@
     </mc:AlternateContent>
     <xdr:clientData/>
   </xdr:oneCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>36</xdr:col>
+      <xdr:colOff>67235</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>134472</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>54</xdr:col>
+      <xdr:colOff>152602</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>112060</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7B8B7337-AA75-8CE6-EC4B-7E62601D7187}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId7"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="7698441" y="2420472"/>
+          <a:ext cx="3312661" cy="2454088"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -927,7 +980,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{58F02C57-D715-48D1-AE39-2C3FEF5CB072}">
-  <dimension ref="D2:AV27"/>
+  <dimension ref="D2:BJ40"/>
   <sheetFormatPr defaultColWidth="2.42578125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="6" max="7" width="2.85546875" bestFit="1" customWidth="1"/>
@@ -939,15 +992,18 @@
     <col min="31" max="31" width="2.85546875" bestFit="1" customWidth="1"/>
     <col min="32" max="32" width="5.140625" customWidth="1"/>
     <col min="33" max="33" width="5.28515625" customWidth="1"/>
+    <col min="60" max="60" width="3" customWidth="1"/>
+    <col min="61" max="61" width="4.7109375" customWidth="1"/>
+    <col min="62" max="62" width="5.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="4:48" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="4:62" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="K2" s="1"/>
       <c r="M2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="4:48" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="4:62" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="K3" s="1"/>
       <c r="M3">
         <v>0</v>
@@ -971,7 +1027,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="4:48" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="4:62" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="N4" s="4"/>
       <c r="O4" s="6">
         <v>2</v>
@@ -1002,7 +1058,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="4:48" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="4:62" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="N5" s="2"/>
       <c r="O5" s="6">
         <v>4</v>
@@ -1033,7 +1089,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="4:48" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="4:62" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="N6" s="7"/>
       <c r="O6" s="11">
         <v>6</v>
@@ -1065,7 +1121,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="4:48" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="4:62" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="N7" s="2"/>
       <c r="O7" s="6">
         <v>8</v>
@@ -1096,8 +1152,11 @@
         <v>1</v>
       </c>
       <c r="AV7" s="6"/>
-    </row>
-    <row r="8" spans="4:48" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="BI7" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="8" spans="4:62" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="N8" s="8"/>
       <c r="R8" s="9"/>
       <c r="V8">
@@ -1124,8 +1183,14 @@
       <c r="AQ8" s="4"/>
       <c r="AR8" s="6"/>
       <c r="AU8" s="5"/>
-    </row>
-    <row r="9" spans="4:48" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="BI8" t="s">
+        <v>8</v>
+      </c>
+      <c r="BJ8" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="4:62" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="N9">
         <v>10</v>
       </c>
@@ -1158,8 +1223,17 @@
       <c r="AQ9" s="2"/>
       <c r="AR9" s="6"/>
       <c r="AU9" s="2"/>
-    </row>
-    <row r="10" spans="4:48" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="BH9">
+        <v>0</v>
+      </c>
+      <c r="BI9">
+        <v>118</v>
+      </c>
+      <c r="BJ9">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="10" spans="4:62" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="V10">
         <v>6</v>
       </c>
@@ -1186,8 +1260,17 @@
       <c r="AS10" s="3"/>
       <c r="AT10" s="3"/>
       <c r="AU10" s="10"/>
-    </row>
-    <row r="11" spans="4:48" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="BH10">
+        <v>1</v>
+      </c>
+      <c r="BI10">
+        <v>268</v>
+      </c>
+      <c r="BJ10">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="11" spans="4:62" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E11" s="12" t="s">
         <v>4</v>
       </c>
@@ -1220,8 +1303,17 @@
       <c r="AQ11" s="2"/>
       <c r="AR11" s="6"/>
       <c r="AU11" s="2"/>
-    </row>
-    <row r="12" spans="4:48" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="BH11">
+        <v>2</v>
+      </c>
+      <c r="BI11">
+        <v>353</v>
+      </c>
+      <c r="BJ11">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="12" spans="4:62" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D12">
         <v>0</v>
       </c>
@@ -1263,8 +1355,17 @@
       </c>
       <c r="AQ12" s="8"/>
       <c r="AU12" s="9"/>
-    </row>
-    <row r="13" spans="4:48" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="BH12">
+        <v>3</v>
+      </c>
+      <c r="BI12">
+        <v>503</v>
+      </c>
+      <c r="BJ12">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="13" spans="4:62" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D13">
         <v>1</v>
       </c>
@@ -1308,8 +1409,17 @@
       </c>
       <c r="AR13" s="6"/>
       <c r="AV13" s="6"/>
-    </row>
-    <row r="14" spans="4:48" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="BH13">
+        <v>4</v>
+      </c>
+      <c r="BI13">
+        <v>148</v>
+      </c>
+      <c r="BJ13">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="14" spans="4:62" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D14">
         <v>2</v>
       </c>
@@ -1351,8 +1461,17 @@
       <c r="AH14" s="13">
         <v>1</v>
       </c>
-    </row>
-    <row r="15" spans="4:48" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="BH14">
+        <v>5</v>
+      </c>
+      <c r="BI14">
+        <v>238</v>
+      </c>
+      <c r="BJ14">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="15" spans="4:62" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D15">
         <v>3</v>
       </c>
@@ -1395,8 +1514,17 @@
       <c r="AH15" s="13">
         <v>1</v>
       </c>
-    </row>
-    <row r="16" spans="4:48" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="BH15">
+        <v>6</v>
+      </c>
+      <c r="BI15">
+        <v>383</v>
+      </c>
+      <c r="BJ15">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="16" spans="4:62" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D16">
         <v>4</v>
       </c>
@@ -1429,8 +1557,17 @@
       <c r="AH16" s="13">
         <v>-1</v>
       </c>
-    </row>
-    <row r="17" spans="4:34" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="BH16">
+        <v>7</v>
+      </c>
+      <c r="BI16">
+        <v>473</v>
+      </c>
+      <c r="BJ16">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="17" spans="4:62" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D17">
         <v>5</v>
       </c>
@@ -1457,8 +1594,17 @@
       <c r="AH17" s="13">
         <v>-1</v>
       </c>
-    </row>
-    <row r="18" spans="4:34" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="BH17">
+        <v>8</v>
+      </c>
+      <c r="BI17">
+        <v>148</v>
+      </c>
+      <c r="BJ17">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="18" spans="4:62" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D18">
         <v>6</v>
       </c>
@@ -1491,8 +1637,17 @@
       <c r="AH18" s="13">
         <v>-1</v>
       </c>
-    </row>
-    <row r="19" spans="4:34" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="BH18">
+        <v>9</v>
+      </c>
+      <c r="BI18">
+        <v>238</v>
+      </c>
+      <c r="BJ18">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="19" spans="4:62" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D19">
         <v>7</v>
       </c>
@@ -1517,8 +1672,17 @@
       <c r="AH19" s="13">
         <v>-1</v>
       </c>
-    </row>
-    <row r="20" spans="4:34" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="BH19">
+        <v>10</v>
+      </c>
+      <c r="BI19">
+        <v>383</v>
+      </c>
+      <c r="BJ19">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="20" spans="4:62" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="AE20">
         <v>16</v>
       </c>
@@ -1531,8 +1695,17 @@
       <c r="AH20" s="13">
         <v>-1</v>
       </c>
-    </row>
-    <row r="21" spans="4:34" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="BH20">
+        <v>11</v>
+      </c>
+      <c r="BI20">
+        <v>473</v>
+      </c>
+      <c r="BJ20">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="21" spans="4:62" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="AE21">
         <v>17</v>
       </c>
@@ -1545,8 +1718,17 @@
       <c r="AH21" s="13">
         <v>-1</v>
       </c>
-    </row>
-    <row r="22" spans="4:34" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="BH21">
+        <v>12</v>
+      </c>
+      <c r="BI21">
+        <v>148</v>
+      </c>
+      <c r="BJ21">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="22" spans="4:62" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="AE22">
         <v>18</v>
       </c>
@@ -1559,8 +1741,17 @@
       <c r="AH22" s="13">
         <v>-1</v>
       </c>
-    </row>
-    <row r="23" spans="4:34" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="BH22">
+        <v>13</v>
+      </c>
+      <c r="BI22">
+        <v>238</v>
+      </c>
+      <c r="BJ22">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="23" spans="4:62" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="AE23">
         <v>19</v>
       </c>
@@ -1573,8 +1764,17 @@
       <c r="AH23" s="13">
         <v>-1</v>
       </c>
-    </row>
-    <row r="24" spans="4:34" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="BH23">
+        <v>14</v>
+      </c>
+      <c r="BI23">
+        <v>383</v>
+      </c>
+      <c r="BJ23">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="24" spans="4:62" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="AE24">
         <v>20</v>
       </c>
@@ -1587,8 +1787,17 @@
       <c r="AH24" s="13">
         <v>-1</v>
       </c>
-    </row>
-    <row r="25" spans="4:34" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="BH24">
+        <v>15</v>
+      </c>
+      <c r="BI24">
+        <v>473</v>
+      </c>
+      <c r="BJ24">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="25" spans="4:62" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="AE25">
         <v>21</v>
       </c>
@@ -1601,8 +1810,17 @@
       <c r="AH25" s="13">
         <v>-1</v>
       </c>
-    </row>
-    <row r="26" spans="4:34" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="BH25">
+        <v>16</v>
+      </c>
+      <c r="BI25">
+        <v>148</v>
+      </c>
+      <c r="BJ25">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="26" spans="4:62" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="AE26">
         <v>22</v>
       </c>
@@ -1615,8 +1833,17 @@
       <c r="AH26" s="13">
         <v>-1</v>
       </c>
-    </row>
-    <row r="27" spans="4:34" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="BH26">
+        <v>17</v>
+      </c>
+      <c r="BI26">
+        <v>238</v>
+      </c>
+      <c r="BJ26">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="27" spans="4:62" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="AE27">
         <v>23</v>
       </c>
@@ -1628,6 +1855,158 @@
       </c>
       <c r="AH27" s="13">
         <v>-1</v>
+      </c>
+      <c r="BH27">
+        <v>18</v>
+      </c>
+      <c r="BI27">
+        <v>383</v>
+      </c>
+      <c r="BJ27">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="28" spans="4:62" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="BH28">
+        <v>19</v>
+      </c>
+      <c r="BI28">
+        <v>473</v>
+      </c>
+      <c r="BJ28">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="29" spans="4:62" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="BH29">
+        <v>20</v>
+      </c>
+      <c r="BI29">
+        <v>118</v>
+      </c>
+      <c r="BJ29">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="30" spans="4:62" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="BH30">
+        <v>21</v>
+      </c>
+      <c r="BI30">
+        <v>268</v>
+      </c>
+      <c r="BJ30">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="31" spans="4:62" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="BH31">
+        <v>22</v>
+      </c>
+      <c r="BI31">
+        <v>353</v>
+      </c>
+      <c r="BJ31">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="32" spans="4:62" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="BH32">
+        <v>23</v>
+      </c>
+      <c r="BI32">
+        <v>503</v>
+      </c>
+      <c r="BJ32">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="33" spans="60:62" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="BH33">
+        <v>24</v>
+      </c>
+      <c r="BI33">
+        <v>150</v>
+      </c>
+      <c r="BJ33">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="34" spans="60:62" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="BH34">
+        <v>25</v>
+      </c>
+      <c r="BI34">
+        <v>239</v>
+      </c>
+      <c r="BJ34">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="35" spans="60:62" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="BH35">
+        <v>26</v>
+      </c>
+      <c r="BI35">
+        <v>150</v>
+      </c>
+      <c r="BJ35">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="36" spans="60:62" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="BH36">
+        <v>27</v>
+      </c>
+      <c r="BI36">
+        <v>239</v>
+      </c>
+      <c r="BJ36">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="37" spans="60:62" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="BH37">
+        <v>28</v>
+      </c>
+      <c r="BI37">
+        <v>120</v>
+      </c>
+      <c r="BJ37">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="38" spans="60:62" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="BH38">
+        <v>29</v>
+      </c>
+      <c r="BI38">
+        <v>148</v>
+      </c>
+      <c r="BJ38">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="39" spans="60:62" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="BH39">
+        <v>30</v>
+      </c>
+      <c r="BI39">
+        <v>120</v>
+      </c>
+      <c r="BJ39">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="40" spans="60:62" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="BH40">
+        <v>31</v>
+      </c>
+      <c r="BI40">
+        <v>148</v>
+      </c>
+      <c r="BJ40">
+        <v>372</v>
       </c>
     </row>
   </sheetData>

</xml_diff>